<commit_message>
Update data files - Bot run at 2026-09-13 14:35:40 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -1082,7 +1082,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-06T14:20:31.526989+00:00</t>
+          <t>2026-09-13T14:35:36.771219+00:00</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1100,7 +1100,7 @@
         <v>63</v>
       </c>
       <c r="J12" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-19 00:57:49 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -1534,7 +1534,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-14T00:41:06.408892+00:00</t>
+          <t>2026-09-19T00:57:45.269107+00:00</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1546,13 +1546,13 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I20" t="n">
         <v>4</v>
       </c>
       <c r="J20" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>[10479, 10503, 10516, 10521, 10555, 10947, 10949, 10957, 10959, 10962, 10967, 10976, 10999, 11005, 11015, 11011, 11033]</t>
+          <t>[10479, 10503, 10516, 10521, 10555, 10947, 10949, 10957, 10959, 10962, 10967, 10976, 10999, 11005, 11015, 11011, 11033, 11044]</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-19 05:29:47 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -1929,7 +1929,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-09-14T05:45:06.622570+00:00</t>
+          <t>2026-09-19T05:29:41.262528+00:00</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1941,13 +1941,13 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I27" t="n">
         <v>16</v>
       </c>
       <c r="J27" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>[7226, 7227, 7223, 7225, 7458, 7692, 7940, 8071, 8191, 8715, 8841, 8977, 9102, 9113, 9190, 9212, 9229, 9245, 9363, 9374, 9372, 9411, 9412, 9447, 9462, 9482, 9477, 9487, 9643, 10378, 10386, 10397, 10403, 10470, 10570, 10573, 10576, 10586, 10585, 10583, 10591, 10589, 10593, 10588, 10597, 10608]</t>
+          <t>[7226, 7227, 7223, 7225, 7458, 7692, 7940, 8071, 8191, 8715, 8841, 8977, 9102, 9113, 9190, 9212, 9229, 9245, 9363, 9374, 9372, 9411, 9412, 9447, 9462, 9482, 9477, 9487, 9643, 10378, 10386, 10397, 10403, 10470, 10570, 10573, 10576, 10586, 10585, 10583, 10591, 10589, 10593, 10588, 10597, 10608, 10617]</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-22 01:46:17 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -1591,7 +1591,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-11T01:21:50.686548+00:00</t>
+          <t>2026-09-22T01:46:09.445754+00:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1609,7 +1609,7 @@
         <v>7</v>
       </c>
       <c r="J21" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-22 12:47:50 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -968,7 +968,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-07T12:55:12.196314+00:00</t>
+          <t>2026-09-22T12:47:40.400184+00:00</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -980,7 +980,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -995,7 +995,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>[24555, 24554, 24559, 24550, 24560, 24556, 24581, 24583, 24587, 24601, 24610, 24613, 24630, 24619, 24633, 24621, 24665, 24661, 24667, 24670, 24660, 24672, 24674, 24683, 24675, 24686, 24697, 24700, 24706, 24653, 24710, 24656, 24658, 24716, 24722, 24717, 24718, 24727, 24719, 24724, 24728, 24725, 24730, 24742, 24735, 24743, 24750, 24756, 24757, 24769, 24770, 24786, 24787, 24796, 24801, 24811, 24823, 24824, 24827, 24830, 24805, 24851, 24839, 24840, 24843, 24847, 24858, 24848, 24875, 24887, 24862, 24890, 24888, 24893, 24894, 24870, 24900, 24899, 24897, 24908, 24913]</t>
+          <t>[24555, 24554, 24559, 24550, 24560, 24556, 24581, 24583, 24587, 24601, 24610, 24613, 24630, 24619, 24633, 24621, 24665, 24661, 24667, 24670, 24660, 24672, 24674, 24683, 24675, 24686, 24697, 24700, 24706, 24653, 24710, 24656, 24658, 24716, 24722, 24717, 24718, 24727, 24719, 24724, 24728, 24725, 24730, 24742, 24735, 24743, 24750, 24756, 24757, 24769, 24770, 24786, 24787, 24796, 24801, 24811, 24823, 24824, 24827, 24830, 24805, 24851, 24839, 24840, 24843, 24847, 24858, 24848, 24875, 24887, 24862, 24890, 24888, 24893, 24894, 24870, 24900, 24899, 24897, 24908, 24913, 24919]</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-23 01:40:16 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -1591,7 +1591,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-22T01:46:09.445754+00:00</t>
+          <t>2026-09-23T01:40:08.060684+00:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1603,7 +1603,7 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I21" t="n">
         <v>7</v>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>[2375, 2380, 2385, 2379, 2387, 2399, 2404, 2406, 2419, 2415, 2428, 2437, 2443, 2449, 2465, 2521, 2871, 2998, 3030, 3051, 3065, 3075, 3449, 3453, 3455, 3458, 3465]</t>
+          <t>[2375, 2380, 2385, 2379, 2387, 2399, 2404, 2406, 2419, 2415, 2428, 2437, 2443, 2449, 2465, 2521, 2871, 2998, 3030, 3051, 3065, 3075, 3449, 3453, 3455, 3458, 3465, 3481]</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-04 12:44:13 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -968,7 +968,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-22T12:47:40.400184+00:00</t>
+          <t>2026-10-04T12:44:03.999720+00:00</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -980,7 +980,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -995,7 +995,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>[24555, 24554, 24559, 24550, 24560, 24556, 24581, 24583, 24587, 24601, 24610, 24613, 24630, 24619, 24633, 24621, 24665, 24661, 24667, 24670, 24660, 24672, 24674, 24683, 24675, 24686, 24697, 24700, 24706, 24653, 24710, 24656, 24658, 24716, 24722, 24717, 24718, 24727, 24719, 24724, 24728, 24725, 24730, 24742, 24735, 24743, 24750, 24756, 24757, 24769, 24770, 24786, 24787, 24796, 24801, 24811, 24823, 24824, 24827, 24830, 24805, 24851, 24839, 24840, 24843, 24847, 24858, 24848, 24875, 24887, 24862, 24890, 24888, 24893, 24894, 24870, 24900, 24899, 24897, 24908, 24913, 24919]</t>
+          <t>[24555, 24554, 24559, 24550, 24560, 24556, 24581, 24583, 24587, 24601, 24610, 24613, 24630, 24619, 24633, 24621, 24665, 24661, 24667, 24670, 24660, 24672, 24674, 24683, 24675, 24686, 24697, 24700, 24706, 24653, 24710, 24656, 24658, 24716, 24722, 24717, 24718, 24727, 24719, 24724, 24728, 24725, 24730, 24742, 24735, 24743, 24750, 24756, 24757, 24769, 24770, 24786, 24787, 24796, 24801, 24811, 24823, 24824, 24827, 24830, 24805, 24851, 24839, 24840, 24843, 24847, 24858, 24848, 24875, 24887, 24862, 24890, 24888, 24893, 24894, 24870, 24900, 24899, 24897, 24908, 24913, 24919, 24942]</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-07 04:03:41 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -1815,7 +1815,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-08-25T04:09:50.096254+00:00</t>
+          <t>2026-10-07T04:03:37.534192+00:00</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1827,13 +1827,13 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I25" t="n">
         <v>15</v>
       </c>
       <c r="J25" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>[2554, 2549, 2561, 2552, 2540, 2545, 2563, 2571, 2599, 2600, 2607, 2628, 2657, 2659, 2665, 2726, 2680, 2777, 2786, 2789, 2790, 2791, 2787, 2793, 2795, 2797, 2803, 2813]</t>
+          <t>[2554, 2549, 2561, 2552, 2540, 2545, 2563, 2571, 2599, 2600, 2607, 2628, 2657, 2659, 2665, 2726, 2680, 2777, 2786, 2789, 2790, 2791, 2787, 2793, 2795, 2797, 2803, 2813, 2834]</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-09 01:44:01 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -1591,7 +1591,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-29T01:27:54.397787+00:00</t>
+          <t>2026-10-09T01:43:57.344224+00:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1603,13 +1603,13 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I21" t="n">
         <v>7</v>
       </c>
       <c r="J21" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>[2375, 2380, 2385, 2379, 2387, 2399, 2404, 2406, 2419, 2415, 2428, 2437, 2443, 2449, 2465, 2521, 2871, 2998, 3030, 3051, 3065, 3075, 3449, 3453, 3455, 3458, 3465, 3481, 3480]</t>
+          <t>[2375, 2380, 2385, 2379, 2387, 2399, 2404, 2406, 2419, 2415, 2428, 2437, 2443, 2449, 2465, 2521, 2871, 2998, 3030, 3051, 3065, 3075, 3449, 3453, 3455, 3458, 3465, 3481, 3480, 3486]</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-11 13:17:01 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -968,7 +968,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-04T12:44:03.999720+00:00</t>
+          <t>2026-10-11T13:16:53.396812+00:00</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -980,7 +980,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -995,7 +995,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>[24555, 24554, 24559, 24550, 24560, 24556, 24581, 24583, 24587, 24601, 24610, 24613, 24630, 24619, 24633, 24621, 24665, 24661, 24667, 24670, 24660, 24672, 24674, 24683, 24675, 24686, 24697, 24700, 24706, 24653, 24710, 24656, 24658, 24716, 24722, 24717, 24718, 24727, 24719, 24724, 24728, 24725, 24730, 24742, 24735, 24743, 24750, 24756, 24757, 24769, 24770, 24786, 24787, 24796, 24801, 24811, 24823, 24824, 24827, 24830, 24805, 24851, 24839, 24840, 24843, 24847, 24858, 24848, 24875, 24887, 24862, 24890, 24888, 24893, 24894, 24870, 24900, 24899, 24897, 24908, 24913, 24919, 24942]</t>
+          <t>[24555, 24554, 24559, 24550, 24560, 24556, 24581, 24583, 24587, 24601, 24610, 24613, 24630, 24619, 24633, 24621, 24665, 24661, 24667, 24670, 24660, 24672, 24674, 24683, 24675, 24686, 24697, 24700, 24706, 24653, 24710, 24656, 24658, 24716, 24722, 24717, 24718, 24727, 24719, 24724, 24728, 24725, 24730, 24742, 24735, 24743, 24750, 24756, 24757, 24769, 24770, 24786, 24787, 24796, 24801, 24811, 24823, 24824, 24827, 24830, 24805, 24851, 24839, 24840, 24843, 24847, 24858, 24848, 24875, 24887, 24862, 24890, 24888, 24893, 24894, 24870, 24900, 24899, 24897, 24908, 24913, 24919, 24942, 24936]</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-13 12:53:55 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -968,7 +968,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-11T13:16:53.396812+00:00</t>
+          <t>2026-10-13T12:53:41.731324+00:00</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -980,7 +980,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -995,7 +995,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>[24555, 24554, 24559, 24550, 24560, 24556, 24581, 24583, 24587, 24601, 24610, 24613, 24630, 24619, 24633, 24621, 24665, 24661, 24667, 24670, 24660, 24672, 24674, 24683, 24675, 24686, 24697, 24700, 24706, 24653, 24710, 24656, 24658, 24716, 24722, 24717, 24718, 24727, 24719, 24724, 24728, 24725, 24730, 24742, 24735, 24743, 24750, 24756, 24757, 24769, 24770, 24786, 24787, 24796, 24801, 24811, 24823, 24824, 24827, 24830, 24805, 24851, 24839, 24840, 24843, 24847, 24858, 24848, 24875, 24887, 24862, 24890, 24888, 24893, 24894, 24870, 24900, 24899, 24897, 24908, 24913, 24919, 24942, 24936]</t>
+          <t>[24555, 24554, 24559, 24550, 24560, 24556, 24581, 24583, 24587, 24601, 24610, 24613, 24630, 24619, 24633, 24621, 24665, 24661, 24667, 24670, 24660, 24672, 24674, 24683, 24675, 24686, 24697, 24700, 24706, 24653, 24710, 24656, 24658, 24716, 24722, 24717, 24718, 24727, 24719, 24724, 24728, 24725, 24730, 24742, 24735, 24743, 24750, 24756, 24757, 24769, 24770, 24786, 24787, 24796, 24801, 24811, 24823, 24824, 24827, 24830, 24805, 24851, 24839, 24840, 24843, 24847, 24858, 24848, 24875, 24887, 24862, 24890, 24888, 24893, 24894, 24870, 24900, 24899, 24897, 24908, 24913, 24919, 24942, 24936, 24928]</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-15 05:33:18 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -1929,7 +1929,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-09-19T05:29:41.262528+00:00</t>
+          <t>2026-10-15T05:33:14.662095+00:00</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1941,13 +1941,13 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I27" t="n">
         <v>16</v>
       </c>
       <c r="J27" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>[7226, 7227, 7223, 7225, 7458, 7692, 7940, 8071, 8191, 8715, 8841, 8977, 9102, 9113, 9190, 9212, 9229, 9245, 9363, 9374, 9372, 9411, 9412, 9447, 9462, 9482, 9477, 9487, 9643, 10378, 10386, 10397, 10403, 10470, 10570, 10573, 10576, 10586, 10585, 10583, 10591, 10589, 10593, 10588, 10597, 10608, 10617]</t>
+          <t>[7226, 7227, 7223, 7225, 7458, 7692, 7940, 8071, 8191, 8715, 8841, 8977, 9102, 9113, 9190, 9212, 9229, 9245, 9363, 9374, 9372, 9411, 9412, 9447, 9462, 9482, 9477, 9487, 9643, 10378, 10386, 10397, 10403, 10470, 10570, 10573, 10576, 10586, 10585, 10583, 10591, 10589, 10593, 10588, 10597, 10608, 10617, 10622]</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-16 01:00:50 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -1534,7 +1534,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-10-15T00:44:17.334827+00:00</t>
+          <t>2026-10-16T01:00:43.746903+00:00</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1552,7 +1552,7 @@
         <v>4</v>
       </c>
       <c r="J20" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-17 12:51:56 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -968,7 +968,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-13T12:53:41.731324+00:00</t>
+          <t>2026-10-17T12:51:42.588573+00:00</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -980,7 +980,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -995,7 +995,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>[24555, 24554, 24559, 24550, 24560, 24556, 24581, 24583, 24587, 24601, 24610, 24613, 24630, 24619, 24633, 24621, 24665, 24661, 24667, 24670, 24660, 24672, 24674, 24683, 24675, 24686, 24697, 24700, 24706, 24653, 24710, 24656, 24658, 24716, 24722, 24717, 24718, 24727, 24719, 24724, 24728, 24725, 24730, 24742, 24735, 24743, 24750, 24756, 24757, 24769, 24770, 24786, 24787, 24796, 24801, 24811, 24823, 24824, 24827, 24830, 24805, 24851, 24839, 24840, 24843, 24847, 24858, 24848, 24875, 24887, 24862, 24890, 24888, 24893, 24894, 24870, 24900, 24899, 24897, 24908, 24913, 24919, 24942, 24936, 24928]</t>
+          <t>[24555, 24554, 24559, 24550, 24560, 24556, 24581, 24583, 24587, 24601, 24610, 24613, 24630, 24619, 24633, 24621, 24665, 24661, 24667, 24670, 24660, 24672, 24674, 24683, 24675, 24686, 24697, 24700, 24706, 24653, 24710, 24656, 24658, 24716, 24722, 24717, 24718, 24727, 24719, 24724, 24728, 24725, 24730, 24742, 24735, 24743, 24750, 24756, 24757, 24769, 24770, 24786, 24787, 24796, 24801, 24811, 24823, 24824, 24827, 24830, 24805, 24851, 24839, 24840, 24843, 24847, 24858, 24848, 24875, 24887, 24862, 24890, 24888, 24893, 24894, 24870, 24900, 24899, 24897, 24908, 24913, 24919, 24942, 24936, 24928, 24953]</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-18 01:22:50 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -1591,7 +1591,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-10-09T01:43:57.344224+00:00</t>
+          <t>2026-10-18T01:22:46.662308+00:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1609,7 +1609,7 @@
         <v>7</v>
       </c>
       <c r="J21" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-20 01:32:21 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -1591,7 +1591,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-10-18T01:22:46.662308+00:00</t>
+          <t>2026-10-20T01:32:14.561146+00:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1603,13 +1603,13 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I21" t="n">
         <v>7</v>
       </c>
       <c r="J21" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>[2375, 2380, 2385, 2379, 2387, 2399, 2404, 2406, 2419, 2415, 2428, 2437, 2443, 2449, 2465, 2521, 2871, 2998, 3030, 3051, 3065, 3075, 3449, 3453, 3455, 3458, 3465, 3481, 3480, 3486]</t>
+          <t>[2375, 2380, 2385, 2379, 2387, 2399, 2404, 2406, 2419, 2415, 2428, 2437, 2443, 2449, 2465, 2521, 2871, 2998, 3030, 3051, 3065, 3075, 3449, 3453, 3455, 3458, 3465, 3481, 3480, 3486, 3497]</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-21 12:47:51 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -968,7 +968,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-17T12:51:42.588573+00:00</t>
+          <t>2026-10-21T12:47:41.616982+00:00</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -980,7 +980,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -995,7 +995,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>[24555, 24554, 24559, 24550, 24560, 24556, 24581, 24583, 24587, 24601, 24610, 24613, 24630, 24619, 24633, 24621, 24665, 24661, 24667, 24670, 24660, 24672, 24674, 24683, 24675, 24686, 24697, 24700, 24706, 24653, 24710, 24656, 24658, 24716, 24722, 24717, 24718, 24727, 24719, 24724, 24728, 24725, 24730, 24742, 24735, 24743, 24750, 24756, 24757, 24769, 24770, 24786, 24787, 24796, 24801, 24811, 24823, 24824, 24827, 24830, 24805, 24851, 24839, 24840, 24843, 24847, 24858, 24848, 24875, 24887, 24862, 24890, 24888, 24893, 24894, 24870, 24900, 24899, 24897, 24908, 24913, 24919, 24942, 24936, 24928, 24953]</t>
+          <t>[24555, 24554, 24559, 24550, 24560, 24556, 24581, 24583, 24587, 24601, 24610, 24613, 24630, 24619, 24633, 24621, 24665, 24661, 24667, 24670, 24660, 24672, 24674, 24683, 24675, 24686, 24697, 24700, 24706, 24653, 24710, 24656, 24658, 24716, 24722, 24717, 24718, 24727, 24719, 24724, 24728, 24725, 24730, 24742, 24735, 24743, 24750, 24756, 24757, 24769, 24770, 24786, 24787, 24796, 24801, 24811, 24823, 24824, 24827, 24830, 24805, 24851, 24839, 24840, 24843, 24847, 24858, 24848, 24875, 24887, 24862, 24890, 24888, 24893, 24894, 24870, 24900, 24899, 24897, 24908, 24913, 24919, 24942, 24936, 24928, 24953, 24963]</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-23 01:12:03 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -1534,7 +1534,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-10-19T00:46:49.040726+00:00</t>
+          <t>2026-10-23T01:11:58.040898+00:00</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1546,7 +1546,7 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I20" t="n">
         <v>4</v>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>[10479, 10503, 10516, 10521, 10555, 10947, 10949, 10957, 10959, 10962, 10967, 10976, 10999, 11005, 11015, 11011, 11033, 11044, 11076]</t>
+          <t>[10479, 10503, 10516, 10521, 10555, 10947, 10949, 10957, 10959, 10962, 10967, 10976, 10999, 11005, 11015, 11011, 11033, 11044, 11076, 11124]</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-24 01:49:46 UTC
</commit_message>
<xml_diff>
--- a/group_promotion_service/data/groups_progress.xlsx
+++ b/group_promotion_service/data/groups_progress.xlsx
@@ -1591,7 +1591,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-10-21T01:51:05.862563+00:00</t>
+          <t>2026-10-24T01:49:40.434555+00:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1603,13 +1603,13 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I21" t="n">
         <v>7</v>
       </c>
       <c r="J21" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>[2375, 2380, 2385, 2379, 2387, 2399, 2404, 2406, 2419, 2415, 2428, 2437, 2443, 2449, 2465, 2521, 2871, 2998, 3030, 3051, 3065, 3075, 3449, 3453, 3455, 3458, 3465, 3481, 3480, 3486, 3497]</t>
+          <t>[2375, 2380, 2385, 2379, 2387, 2399, 2404, 2406, 2419, 2415, 2428, 2437, 2443, 2449, 2465, 2521, 2871, 2998, 3030, 3051, 3065, 3075, 3449, 3453, 3455, 3458, 3465, 3481, 3480, 3486, 3497, 3522]</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">

</xml_diff>